<commit_message>
Add button-based file upload test
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ABHISHEK\eclipse-workspace\selenium-framework\src\test\resources\testData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ABHISHEK\eclipse-workspace\Data-Driven-Framework\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{563ED220-54FC-41BC-8C28-B6F6666A4788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDE1E1B5-3512-4763-8E84-5D0F5F6E1060}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0CE966F4-9799-4302-B101-6A8B30663B20}"/>
+    <workbookView xWindow="960" yWindow="0" windowWidth="22080" windowHeight="12240" activeTab="1" xr2:uid="{0CE966F4-9799-4302-B101-6A8B30663B20}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
+    <sheet name="UploadFiles" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>username</t>
   </si>
@@ -48,6 +49,12 @@
   </si>
   <si>
     <t>pwd</t>
+  </si>
+  <si>
+    <t>FileName</t>
+  </si>
+  <si>
+    <t>TestPdf.pdf</t>
   </si>
 </sst>
 </file>
@@ -441,4 +448,24 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56013896-E995-4332-8747-DA8B3CE51FA7}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Configure framework for parallel test execution
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ABHISHEK\eclipse-workspace\Data-Driven-Framework\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDE1E1B5-3512-4763-8E84-5D0F5F6E1060}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83703D02-399D-4054-BA23-39053C632962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="960" yWindow="0" windowWidth="22080" windowHeight="12240" activeTab="1" xr2:uid="{0CE966F4-9799-4302-B101-6A8B30663B20}"/>
+    <workbookView xWindow="960" yWindow="0" windowWidth="22080" windowHeight="12240" xr2:uid="{0CE966F4-9799-4302-B101-6A8B30663B20}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
   <si>
     <t>username</t>
   </si>
@@ -55,6 +55,9 @@
   </si>
   <si>
     <t>TestPdf.pdf</t>
+  </si>
+  <si>
+    <t>pwdd</t>
   </si>
 </sst>
 </file>
@@ -426,7 +429,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A1D7EA8-9234-4640-A8CF-76388E869F89}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -445,6 +448,14 @@
         <v>3</v>
       </c>
     </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -454,6 +465,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56013896-E995-4332-8747-DA8B3CE51FA7}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">

</xml_diff>